<commit_message>
Agent 3: carry-forward code and exclusive-option checks
</commit_message>
<xml_diff>
--- a/out/S01_campus_cafeteria_experience/agent3/agent3_test_cases_for_review.xlsx
+++ b/out/S01_campus_cafeteria_experience/agent3/agent3_test_cases_for_review.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2222,30 +2222,217 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Q6 | Please describe the main problem. | text | — | Show if: Q5 == 'Yes'
+Validate: {"min_length": 10, "max_length": 500}</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>TC-ad86701f00</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Prove Q6 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at least 10 characters; the answer must be at most 500 characters</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>1. S1 = Yes
+2. S2 = Yes
+3. Q1 = Counter
+4. Q2 = Very poor
+5. Q3 = Very poor
+6. Q4 = Food quality
+7. Q5 = Yes</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>At Q6, type a 500-character answer, then submit.</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>1. the survey ACCEPTS the answer and moves to the next page</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Answer rule accepts or rejects</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Q6 | Please describe the main problem. | text | — | Show if: Q5 == 'Yes'
+Validate: {"min_length": 10, "max_length": 500}</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>TC-566303fa26</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Prove Q6 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at least 10 characters; the answer must be at most 500 characters</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>1. S1 = Yes
+2. S2 = Yes
+3. Q1 = Counter
+4. Q2 = Very poor
+5. Q3 = Very poor
+6. Q4 = Food quality
+7. Q5 = Yes</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>At Q6, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>1. the survey ACCEPTS the answer and moves to the next page</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Answer rule accepts or rejects</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Q6 | Please describe the main problem. | text | — | Show if: Q5 == 'Yes'
+Validate: {"min_length": 10, "max_length": 500}</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>TC-2587d31b15</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Prove Q6 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a text question</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>1. S1 = Yes
+2. S2 = Yes
+3. Q1 = Counter
+4. Q2 = Very poor
+5. Q3 = Very poor
+6. Q4 = Food quality
+7. Q5 = Yes</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>At Q6, type 3 spaces and nothing else, then submit.</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>1. the survey REFUSES to move on; the same page reappears
+2. an error message is shown against Q6</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Blank answer is blocked</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
           <t>Q7</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>Q7 | How likely are you to recommend this service? | single | 0; 1; 2; 3; 4; 5; 6; 7; 8; 9; 10 | Always show</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>TC-6a0410fc63</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Prove the survey flows correctly at Q7: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Yes
@@ -2258,58 +2445,58 @@
 9. Q7 = 0</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>1. Q7 IS shown on the page
 2. the next question shown is Q8</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Shows / hides correctly</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Q7</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Q7 | How likely are you to recommend this service? | single | 0; 1; 2; 3; 4; 5; 6; 7; 8; 9; 10 | Always show</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>TC-3af13688c6</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>Prove Q7 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a single question</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Yes
@@ -2321,59 +2508,59 @@
 8. Q6 = xxxxxxxxxx</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>At Q7, select nothing at all, then submit.</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>1. the survey REFUSES to move on; the same page reappears
 2. an error message is shown against Q7</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>Blank answer is blocked</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Q8 | What is the single most important improvement you would suggest? | text | — | Validate: {"max_length": 500}
 Optional</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>TC-6452a460af</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Prove the survey flows correctly at Q8: answer it normally and the respondent should move on to whatever the questionnaire says comes next, not stop or jump elsewhere</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Yes
@@ -2386,59 +2573,59 @@
 9. Q7 = 0</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>1. Q8 IS shown on the page
 2. the respondent reaches the normal thank-you page</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>Shows / hides correctly</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Q8 | What is the single most important improvement you would suggest? | text | — | Validate: {"max_length": 500}
 Optional</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>TC-785a9414c4</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>Prove Q8 ACCEPTS an answer that obeys its rule. The QRE's rule is: the answer must be at most 500 characters</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Yes
@@ -2451,58 +2638,58 @@
 9. Q7 = 0</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>At Q8, type “x”, then submit.</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
+      <c r="I36" s="3" t="inlineStr">
         <is>
           <t>1. the survey ACCEPTS the answer and moves to the next page</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>Answer rule accepts or rejects</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Q8 | What is the single most important improvement you would suggest? | text | — | Validate: {"max_length": 500}
 Optional</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>TC-12b005a4ef</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>Prove Q8 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at most 500 characters</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Yes
@@ -2515,59 +2702,59 @@
 9. Q7 = 0</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>At Q8, type a 501-character answer, then submit.</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>1. the survey REFUSES to move on; the same page reappears
 2. an error message is shown against Q8</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>Answer rule accepts or rejects</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Q8 | What is the single most important improvement you would suggest? | text | — | Validate: {"max_length": 500}
 Optional</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>TC-35736daef1</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>Prove Q8 lets the respondent through with no answer, because the questionnaire marks it optional</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Yes
@@ -2580,53 +2767,58 @@
 9. Q7 = 0</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>At Q8, type nothing, then submit.</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>1. the survey ACCEPTS the answer and moves to the next page</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Blank answer is blocked</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>whole survey</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>TC-6b6c46c5df</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>Prove the survey finishes normally for a respondent who answers everything and triggers no screen-out</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Q8 | What is the single most important improvement you would suggest? | text | — | Validate: {"max_length": 500}
+Optional</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>TC-75945e73bd</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Prove Q8 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at most 500 characters</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>1. S1 = Yes
 2. S2 = Yes
@@ -2639,22 +2831,209 @@
 9. Q7 = 0</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>At Q8, type a 500-character answer, then submit.</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>1. the survey ACCEPTS the answer and moves to the next page</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Answer rule accepts or rejects</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Q8 | What is the single most important improvement you would suggest? | text | — | Validate: {"max_length": 500}
+Optional</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>TC-4d9f269943</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Prove Q8 REJECTS an answer that breaks its rule. The QRE's rule is: the answer must be at most 500 characters</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>1. S1 = Yes
+2. S2 = Yes
+3. Q1 = Counter
+4. Q2 = Very poor
+5. Q3 = Very poor
+6. Q4 = Food quality
+7. Q5 = Yes
+8. Q6 = xxxxxxxxxx
+9. Q7 = 0</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>At Q8, type “O'Brien said "yes" &lt;50% &amp; more”, then submit.</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>1. the survey ACCEPTS the answer and moves to the next page</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Answer rule accepts or rejects</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Q8 | What is the single most important improvement you would suggest? | text | — | Validate: {"max_length": 500}
+Optional</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>TC-a7509385dc</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Prove Q8 refuses to let the respondent past when it is left blank. The questionnaire marks it compulsory, and it is a text question</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>1. S1 = Yes
+2. S2 = Yes
+3. Q1 = Counter
+4. Q2 = Very poor
+5. Q3 = Very poor
+6. Q4 = Food quality
+7. Q5 = Yes
+8. Q6 = xxxxxxxxxx
+9. Q7 = 0</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>At Q8, type 3 spaces and nothing else, then submit.</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>1. the survey ACCEPTS the answer and moves to the next page</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Blank answer is blocked</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>whole survey</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>TC-6b6c46c5df</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Prove the survey finishes normally for a respondent who answers everything and triggers no screen-out</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>1. S1 = Yes
+2. S2 = Yes
+3. Q1 = Counter
+4. Q2 = Very poor
+5. Q3 = Very poor
+6. Q4 = Food quality
+7. Q5 = Yes
+8. Q6 = xxxxxxxxxx
+9. Q7 = 0</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
         <is>
           <t>Answer through the whole survey as listed, then observe where it ends.</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr">
+      <c r="I42" s="3" t="inlineStr">
         <is>
           <t>1. the respondent reaches the normal thank-you page</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>Survey ends in the right place</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>